<commit_message>
Define zone colors and add consolidated CAB/DAMA Excel sheet
Caracas Azul Marino, Valencia Vinotinto, Barquisimeto Verde replace generic
additional color. Add Short Playa-style CANTIDADES POR COLORES sheets with
blanco rows first then zone colors by size.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SPOTS_PRODUCCION_EXPANSION.xlsx
+++ b/SPOTS_PRODUCCION_EXPANSION.xlsx
@@ -8,10 +8,12 @@
   </bookViews>
   <sheets>
     <sheet name="RESUMEN" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Caracas" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Valencia" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Barquisimeto" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="TELA" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="CAB" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="DAMA" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Caracas" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Valencia" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Barquisimeto" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="TELA" sheetId="7" state="visible" r:id="rId7"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -54,7 +56,7 @@
       <sz val="11"/>
     </font>
   </fonts>
-  <fills count="5">
+  <fills count="6">
     <fill>
       <patternFill/>
     </fill>
@@ -69,6 +71,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="00E5E7EB"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D1FAE5"/>
       </patternFill>
     </fill>
     <fill>
@@ -103,7 +110,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="11">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -121,7 +128,10 @@
     </xf>
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="6" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -488,7 +498,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D25"/>
+  <dimension ref="A1:D26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -555,189 +565,194 @@
     <row r="7">
       <c r="A7" s="2" t="inlineStr">
         <is>
-          <t>Color adicional</t>
+          <t>Colores zona</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
+          <t>Caracas Azul Marino · Valencia Vinotinto · Barquisimeto Verde</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="2" t="inlineStr">
+        <is>
+          <t>Factor color</t>
+        </is>
+      </c>
+      <c r="B8" t="inlineStr">
+        <is>
           <t>70% del blanco principal</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="3" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="3" t="inlineStr">
         <is>
           <t>Zona</t>
         </is>
       </c>
-      <c r="B9" s="3" t="inlineStr">
+      <c r="B10" s="3" t="inlineStr">
         <is>
           <t>Blanco</t>
         </is>
       </c>
-      <c r="C9" s="3" t="inlineStr">
-        <is>
-          <t>Color adicional</t>
-        </is>
-      </c>
-      <c r="D9" s="3" t="inlineStr">
+      <c r="C10" s="3" t="inlineStr">
+        <is>
+          <t>Color zona</t>
+        </is>
+      </c>
+      <c r="D10" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
-      </c>
-    </row>
-    <row r="10">
-      <c r="A10" s="4" t="inlineStr">
-        <is>
-          <t>CARACAS</t>
-        </is>
-      </c>
-      <c r="B10" s="4" t="n">
-        <v>279</v>
-      </c>
-      <c r="C10" s="4" t="n">
-        <v>196</v>
-      </c>
-      <c r="D10" s="4" t="n">
-        <v>475</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>VALENCIA</t>
+          <t>CARACAS</t>
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>221</v>
-      </c>
-      <c r="C11" s="4" t="n">
-        <v>154</v>
+        <v>279</v>
+      </c>
+      <c r="C11" s="4" t="inlineStr">
+        <is>
+          <t>Azul Marino (196)</t>
+        </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>375</v>
+        <v>475</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
+          <t>VALENCIA</t>
+        </is>
+      </c>
+      <c r="B12" s="4" t="n">
+        <v>221</v>
+      </c>
+      <c r="C12" s="4" t="inlineStr">
+        <is>
+          <t>Vinotinto (154)</t>
+        </is>
+      </c>
+      <c r="D12" s="4" t="n">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="4" t="inlineStr">
+        <is>
           <t>BARQUISIMETO</t>
         </is>
       </c>
-      <c r="B12" s="4" t="n">
+      <c r="B13" s="4" t="n">
         <v>420</v>
       </c>
-      <c r="C12" s="4" t="n">
-        <v>154</v>
-      </c>
-      <c r="D12" s="4" t="n">
+      <c r="C13" s="4" t="inlineStr">
+        <is>
+          <t>Verde (154)</t>
+        </is>
+      </c>
+      <c r="D13" s="4" t="n">
         <v>574</v>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="5" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="5" t="inlineStr">
         <is>
           <t>TOTAL EXPANSIÓN</t>
         </is>
       </c>
-      <c r="B13" s="5" t="n">
+      <c r="B14" s="5" t="n">
         <v>920</v>
       </c>
-      <c r="C13" s="5" t="n">
+      <c r="C14" s="5" t="n">
         <v>504</v>
       </c>
-      <c r="D13" s="5" t="n">
+      <c r="D14" s="5" t="n">
         <v>1424</v>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="2" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="2" t="inlineStr">
         <is>
           <t>Nota metodológica</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>Proyección calibrada 3m · mix talla/género VELA (Jun 26, Jul 26, Ago 26): share género MC · curva talla por género como dashboard Tallas (todo SPOTS). Blanco principal + Color adicional al 70%. Caracas ~475 · Valencia ~375 · Barquisimeto ~574 (Ciudad 220 + Virgen 200 + adicional 154). Solo Manga Corta.</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="7" t="inlineStr">
+    <row r="17">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>Proyección calibrada 3m · mix talla/género VELA (Jun 26, Jul 26, Ago 26): share género MC · curva talla por género como dashboard Tallas (todo SPOTS). Colores zona: Caracas Azul Marino · Valencia Vinotinto · Barquisimeto Verde (70% del blanco principal). Caracas ~475 · Valencia ~375 · Barquisimeto ~574 (Ciudad 220 + Virgen 200 + Verde 154). Solo Manga Corta.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="7" t="inlineStr">
         <is>
           <t>Compra de tela (referencia)</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" t="inlineStr">
+    <row r="20">
+      <c r="A20" t="inlineStr">
         <is>
           <t>Consumo 0.45 kg/und · stock seguridad +20%</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="3" t="inlineStr">
         <is>
           <t>Material</t>
         </is>
       </c>
-      <c r="B20" s="3" t="inlineStr">
+      <c r="B21" s="3" t="inlineStr">
         <is>
           <t>Unidades</t>
         </is>
       </c>
-      <c r="C20" s="3" t="inlineStr">
+      <c r="C21" s="3" t="inlineStr">
         <is>
           <t>Tela (kg)</t>
         </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="4" t="inlineStr">
-        <is>
-          <t>Blanco (total)</t>
-        </is>
-      </c>
-      <c r="B21" s="4" t="n">
-        <v>920</v>
-      </c>
-      <c r="C21" s="4" t="n">
-        <v>497</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>Color adicional — Caracas</t>
+          <t>Blanco (total)</t>
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>196</v>
+        <v>920</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>106</v>
+        <v>497</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>Color adicional — Valencia</t>
+          <t>Azul Marino</t>
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>154</v>
+        <v>196</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>83</v>
+        <v>106</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>Color adicional — Barquisimeto</t>
+          <t>Vinotinto</t>
         </is>
       </c>
       <c r="B24" s="4" t="n">
@@ -748,27 +763,682 @@
       </c>
     </row>
     <row r="25">
-      <c r="A25" s="5" t="inlineStr">
+      <c r="A25" s="4" t="inlineStr">
+        <is>
+          <t>Verde</t>
+        </is>
+      </c>
+      <c r="B25" s="4" t="n">
+        <v>154</v>
+      </c>
+      <c r="C25" s="4" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="5" t="inlineStr">
         <is>
           <t>TOTAL TELA</t>
         </is>
       </c>
-      <c r="B25" s="5" t="n">
+      <c r="B26" s="5" t="n">
         <v>1424</v>
       </c>
-      <c r="C25" s="5" t="n">
+      <c r="C26" s="5" t="n">
         <v>769</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A16:D16"/>
+    <mergeCell ref="A17:D17"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>CANTIDADES POR COLORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>SPOTS MANGA CORTA CAB</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>2XL</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Ciudad · Blanco (Barquisimeto)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>36</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Virgen · Blanco (Barquisimeto)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>27</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>17</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>113</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Caracas · Blanco (Caracas)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>42</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>46</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>8</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>156</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Valencia · Blanco (Valencia)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>37</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>29</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>124</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL BLANCO</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>138</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>152</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>122</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>78</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>26</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>516</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Azul Marino · Caracas</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>30</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>32</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>110</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Vinotinto · Valencia</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Verde · Barquisimeto</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>13</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL COLORES</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>76</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>84</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>66</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>42</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>16</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>284</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>214</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>236</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>188</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>120</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>42</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>800</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="36" customWidth="1" min="1" max="1"/>
+    <col width="8" customWidth="1" min="2" max="2"/>
+    <col width="8" customWidth="1" min="3" max="3"/>
+    <col width="8" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="8" customWidth="1" min="7" max="7"/>
+    <col width="8" customWidth="1" min="8" max="8"/>
+    <col width="8" customWidth="1" min="9" max="9"/>
+    <col width="8" customWidth="1" min="10" max="10"/>
+    <col width="8" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="8" t="inlineStr">
+        <is>
+          <t>CANTIDADES POR COLORES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>SPOTS MANGA CORTA DAMA</t>
+        </is>
+      </c>
+      <c r="B2" s="3" t="inlineStr">
+        <is>
+          <t>XS</t>
+        </is>
+      </c>
+      <c r="C2" s="3" t="inlineStr">
+        <is>
+          <t>S</t>
+        </is>
+      </c>
+      <c r="D2" s="3" t="inlineStr">
+        <is>
+          <t>M</t>
+        </is>
+      </c>
+      <c r="E2" s="3" t="inlineStr">
+        <is>
+          <t>L</t>
+        </is>
+      </c>
+      <c r="F2" s="3" t="inlineStr">
+        <is>
+          <t>XL</t>
+        </is>
+      </c>
+      <c r="G2" s="3" t="inlineStr">
+        <is>
+          <t>Tot</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="4" t="inlineStr">
+        <is>
+          <t>Ciudad · Blanco (Barquisimeto)</t>
+        </is>
+      </c>
+      <c r="B3" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="C3" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="D3" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E3" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F3" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G3" s="4" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Virgen · Blanco (Barquisimeto)</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="C4" s="4" t="n">
+        <v>24</v>
+      </c>
+      <c r="D4" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E4" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F4" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G4" s="4" t="n">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="4" t="inlineStr">
+        <is>
+          <t>Caracas · Blanco (Caracas)</t>
+        </is>
+      </c>
+      <c r="B5" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="C5" s="4" t="n">
+        <v>33</v>
+      </c>
+      <c r="D5" s="4" t="n">
+        <v>35</v>
+      </c>
+      <c r="E5" s="4" t="n">
+        <v>16</v>
+      </c>
+      <c r="F5" s="4" t="n">
+        <v>6</v>
+      </c>
+      <c r="G5" s="4" t="n">
+        <v>123</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="4" t="inlineStr">
+        <is>
+          <t>Valencia · Blanco (Valencia)</t>
+        </is>
+      </c>
+      <c r="B6" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="C6" s="4" t="n">
+        <v>26</v>
+      </c>
+      <c r="D6" s="4" t="n">
+        <v>28</v>
+      </c>
+      <c r="E6" s="4" t="n">
+        <v>12</v>
+      </c>
+      <c r="F6" s="4" t="n">
+        <v>5</v>
+      </c>
+      <c r="G6" s="4" t="n">
+        <v>97</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL BLANCO</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n">
+        <v>108</v>
+      </c>
+      <c r="C7" s="5" t="n">
+        <v>109</v>
+      </c>
+      <c r="D7" s="5" t="n">
+        <v>116</v>
+      </c>
+      <c r="E7" s="5" t="n">
+        <v>51</v>
+      </c>
+      <c r="F7" s="5" t="n">
+        <v>20</v>
+      </c>
+      <c r="G7" s="5" t="n">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>Azul Marino · Caracas</t>
+        </is>
+      </c>
+      <c r="B9" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>23</v>
+      </c>
+      <c r="D9" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="E9" s="4" t="n">
+        <v>11</v>
+      </c>
+      <c r="F9" s="4" t="n">
+        <v>4</v>
+      </c>
+      <c r="G9" s="4" t="n">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="4" t="inlineStr">
+        <is>
+          <t>Vinotinto · Valencia</t>
+        </is>
+      </c>
+      <c r="B10" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="C10" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D10" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="E10" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F10" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G10" s="4" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="4" t="inlineStr">
+        <is>
+          <t>Verde · Barquisimeto</t>
+        </is>
+      </c>
+      <c r="B11" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="C11" s="4" t="n">
+        <v>18</v>
+      </c>
+      <c r="D11" s="4" t="n">
+        <v>19</v>
+      </c>
+      <c r="E11" s="4" t="n">
+        <v>9</v>
+      </c>
+      <c r="F11" s="4" t="n">
+        <v>3</v>
+      </c>
+      <c r="G11" s="4" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>TOTAL COLORES</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="C12" s="5" t="n">
+        <v>59</v>
+      </c>
+      <c r="D12" s="5" t="n">
+        <v>63</v>
+      </c>
+      <c r="E12" s="5" t="n">
+        <v>29</v>
+      </c>
+      <c r="F12" s="5" t="n">
+        <v>10</v>
+      </c>
+      <c r="G12" s="5" t="n">
+        <v>220</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="9" t="inlineStr">
+        <is>
+          <t>TOTAL GENERAL</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="n">
+        <v>167</v>
+      </c>
+      <c r="C13" s="9" t="n">
+        <v>168</v>
+      </c>
+      <c r="D13" s="9" t="n">
+        <v>179</v>
+      </c>
+      <c r="E13" s="9" t="n">
+        <v>80</v>
+      </c>
+      <c r="F13" s="9" t="n">
+        <v>30</v>
+      </c>
+      <c r="G13" s="9" t="n">
+        <v>624</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -798,12 +1468,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Caracas · 4 tiendas CCS (2 alto peso · 1 media · 1 bajo) · MC · Blanco + Color adicional al 70%</t>
+          <t>Caracas · 4 tiendas CCS (2 alto peso · 1 media · 1 bajo) · MC · Blanco + Azul Marino al 70%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>CAB</t>
         </is>
@@ -856,51 +1526,51 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Caracas (Blanco)</t>
+          <t>Caracas (Azul Marino)</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>42</v>
+        <v>30</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>46</v>
+        <v>32</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>37</v>
+        <v>26</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>23</v>
+        <v>16</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>156</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Caracas Alt (Color adicional)</t>
+          <t>Caracas (Blanco)</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>32</v>
+        <v>46</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>26</v>
+        <v>37</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>110</v>
+        <v>156</v>
       </c>
     </row>
     <row r="10">
@@ -929,7 +1599,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>DAMA</t>
         </is>
@@ -982,51 +1652,51 @@
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>Caracas (Blanco)</t>
+          <t>Caracas (Azul Marino)</t>
         </is>
       </c>
       <c r="B15" s="4" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="C15" s="4" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="D15" s="4" t="n">
-        <v>35</v>
+        <v>25</v>
       </c>
       <c r="E15" s="4" t="n">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>123</v>
+        <v>86</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Caracas Alt (Color adicional)</t>
+          <t>Caracas (Blanco)</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>25</v>
+        <v>35</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>86</v>
+        <v>123</v>
       </c>
     </row>
     <row r="17">
@@ -1055,12 +1725,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>TOTAL ZONA CARACAS</t>
         </is>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="11" t="n">
         <v>475</v>
       </c>
     </row>
@@ -1069,7 +1739,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1099,12 +1769,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Valencia · 2 tiendas · MC · Blanco + Color adicional al 70%</t>
+          <t>Valencia · 2 tiendas · MC · Blanco + Vinotinto al 70%</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>CAB</t>
         </is>
@@ -1182,7 +1852,7 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Valencia Alt (Color adicional)</t>
+          <t>Valencia (Vinotinto)</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
@@ -1230,7 +1900,7 @@
       </c>
     </row>
     <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+      <c r="A12" s="10" t="inlineStr">
         <is>
           <t>DAMA</t>
         </is>
@@ -1308,7 +1978,7 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Valencia Alt (Color adicional)</t>
+          <t>Valencia (Vinotinto)</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
@@ -1356,12 +2026,12 @@
       </c>
     </row>
     <row r="19">
-      <c r="A19" s="10" t="inlineStr">
+      <c r="A19" s="11" t="inlineStr">
         <is>
           <t>TOTAL ZONA VALENCIA</t>
         </is>
       </c>
-      <c r="B19" s="10" t="n">
+      <c r="B19" s="11" t="n">
         <v>375</v>
       </c>
     </row>
@@ -1370,7 +2040,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1400,12 +2070,12 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Barquisimeto · 1 tienda · MC · Ciudad 220 + Virgen 200 + Color adicional 154 (70% Ciudad) · total 574</t>
+          <t>Barquisimeto · 1 tienda · MC · Ciudad 220 + Virgen 200 + Verde 154 (70% Ciudad) · total 574</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="9" t="inlineStr">
+      <c r="A5" s="10" t="inlineStr">
         <is>
           <t>CAB</t>
         </is>
@@ -1458,51 +2128,51 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Barquisimeto (Color adicional)</t>
+          <t>Ciudad (Blanco)</t>
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>23</v>
+        <v>33</v>
       </c>
       <c r="C8" s="4" t="n">
-        <v>26</v>
+        <v>36</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>20</v>
+        <v>29</v>
       </c>
       <c r="E8" s="4" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>87</v>
+        <v>123</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Ciudad (Blanco)</t>
+          <t>Ciudad (Verde)</t>
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>33</v>
+        <v>23</v>
       </c>
       <c r="C9" s="4" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>29</v>
+        <v>20</v>
       </c>
       <c r="E9" s="4" t="n">
-        <v>19</v>
+        <v>13</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>123</v>
+        <v>87</v>
       </c>
     </row>
     <row r="10">
@@ -1556,7 +2226,7 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+      <c r="A13" s="10" t="inlineStr">
         <is>
           <t>DAMA</t>
         </is>
@@ -1609,51 +2279,51 @@
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>Barquisimeto (Color adicional)</t>
+          <t>Ciudad (Blanco)</t>
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>18</v>
+        <v>26</v>
       </c>
       <c r="D16" s="4" t="n">
-        <v>19</v>
+        <v>28</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>67</v>
+        <v>97</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>Ciudad (Blanco)</t>
+          <t>Ciudad (Verde)</t>
         </is>
       </c>
       <c r="B17" s="4" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>26</v>
+        <v>18</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>28</v>
+        <v>19</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>97</v>
+        <v>67</v>
       </c>
     </row>
     <row r="18">
@@ -1707,12 +2377,12 @@
       </c>
     </row>
     <row r="21">
-      <c r="A21" s="10" t="inlineStr">
+      <c r="A21" s="11" t="inlineStr">
         <is>
           <t>TOTAL ZONA BARQUISIMETO</t>
         </is>
       </c>
-      <c r="B21" s="10" t="n">
+      <c r="B21" s="11" t="n">
         <v>574</v>
       </c>
     </row>
@@ -1721,7 +2391,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1864,12 +2534,12 @@
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>Color adicional</t>
+          <t>Azul Marino</t>
         </is>
       </c>
       <c r="B7" s="4" t="inlineStr">
         <is>
-          <t>Caracas · Caracas Alt</t>
+          <t>Caracas · Caracas</t>
         </is>
       </c>
       <c r="C7" s="4" t="n">
@@ -1892,12 +2562,12 @@
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>Color adicional</t>
+          <t>Vinotinto</t>
         </is>
       </c>
       <c r="B8" s="4" t="inlineStr">
         <is>
-          <t>Valencia · Valencia Alt</t>
+          <t>Valencia · Valencia</t>
         </is>
       </c>
       <c r="C8" s="4" t="n">
@@ -1920,12 +2590,12 @@
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>Color adicional</t>
+          <t>Verde</t>
         </is>
       </c>
       <c r="B9" s="4" t="inlineStr">
         <is>
-          <t>Barquisimeto · Barquisimeto</t>
+          <t>Barquisimeto · Ciudad</t>
         </is>
       </c>
       <c r="C9" s="4" t="n">

</xml_diff>

<commit_message>
Sync production Excel from manual CAB/DAMA edits across all sheets
Add sync_produccion_xlsx to use CAB/DAMA as source of truth and regenerate
zone sheets, RESUMEN, TELA with corrected subtotals and fabric totals.

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SPOTS_PRODUCCION_EXPANSION.xlsx
+++ b/SPOTS_PRODUCCION_EXPANSION.xlsx
@@ -532,11 +532,7 @@
           <t>Base rotación</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr">
-        <is>
-          <t>Jun 26 · Jul 26 · Ago 26</t>
-        </is>
-      </c>
+      <c r="B4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -615,15 +611,15 @@
         </is>
       </c>
       <c r="B11" s="4" t="n">
-        <v>279</v>
+        <v>283</v>
       </c>
       <c r="C11" s="4" t="inlineStr">
         <is>
-          <t>Azul Marino (196)</t>
+          <t>Azul Marino (209)</t>
         </is>
       </c>
       <c r="D11" s="4" t="n">
-        <v>475</v>
+        <v>492</v>
       </c>
     </row>
     <row r="12">
@@ -633,15 +629,15 @@
         </is>
       </c>
       <c r="B12" s="4" t="n">
-        <v>221</v>
+        <v>228</v>
       </c>
       <c r="C12" s="4" t="inlineStr">
         <is>
-          <t>Vinotinto (154)</t>
+          <t>Vinotinto (174)</t>
         </is>
       </c>
       <c r="D12" s="4" t="n">
-        <v>375</v>
+        <v>402</v>
       </c>
     </row>
     <row r="13">
@@ -651,15 +647,15 @@
         </is>
       </c>
       <c r="B13" s="4" t="n">
-        <v>420</v>
+        <v>441</v>
       </c>
       <c r="C13" s="4" t="inlineStr">
         <is>
-          <t>Verde (154)</t>
+          <t>Verde (175)</t>
         </is>
       </c>
       <c r="D13" s="4" t="n">
-        <v>574</v>
+        <v>616</v>
       </c>
     </row>
     <row r="14">
@@ -669,13 +665,13 @@
         </is>
       </c>
       <c r="B14" s="5" t="n">
-        <v>920</v>
+        <v>952</v>
       </c>
       <c r="C14" s="5" t="n">
-        <v>504</v>
+        <v>558</v>
       </c>
       <c r="D14" s="5" t="n">
-        <v>1424</v>
+        <v>1510</v>
       </c>
     </row>
     <row r="16">
@@ -688,7 +684,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Proyección calibrada 3m · mix talla/género VELA (Jun 26, Jul 26, Ago 26): share género MC · curva talla por género como dashboard Tallas (todo SPOTS). Colores zona: Caracas Azul Marino · Valencia Vinotinto · Barquisimeto Verde (70% del blanco principal). Caracas ~475 · Valencia ~375 · Barquisimeto ~574 (Ciudad 220 + Virgen 200 + Verde 154). Solo Manga Corta.</t>
+          <t>Cantidades ajustadas manualmente · horizonte 3 meses · colores: Caracas Azul Marino · Valencia Vinotinto · Barquisimeto Verde.</t>
         </is>
       </c>
     </row>
@@ -730,10 +726,10 @@
         </is>
       </c>
       <c r="B22" s="4" t="n">
-        <v>920</v>
+        <v>952</v>
       </c>
       <c r="C22" s="4" t="n">
-        <v>497</v>
+        <v>514</v>
       </c>
     </row>
     <row r="23">
@@ -743,10 +739,10 @@
         </is>
       </c>
       <c r="B23" s="4" t="n">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="C23" s="4" t="n">
-        <v>106</v>
+        <v>113</v>
       </c>
     </row>
     <row r="24">
@@ -756,10 +752,10 @@
         </is>
       </c>
       <c r="B24" s="4" t="n">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="C24" s="4" t="n">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="25">
@@ -769,10 +765,10 @@
         </is>
       </c>
       <c r="B25" s="4" t="n">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="C25" s="4" t="n">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="26">
@@ -782,10 +778,10 @@
         </is>
       </c>
       <c r="B26" s="5" t="n">
-        <v>1424</v>
+        <v>1510</v>
       </c>
       <c r="C26" s="5" t="n">
-        <v>769</v>
+        <v>815</v>
       </c>
     </row>
   </sheetData>
@@ -881,10 +877,10 @@
         <v>19</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="4">
@@ -906,10 +902,10 @@
         <v>17</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="5">
@@ -931,10 +927,10 @@
         <v>23</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="6">
@@ -956,10 +952,10 @@
         <v>19</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="7">
@@ -981,10 +977,10 @@
         <v>78</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>26</v>
+        <v>40</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>516</v>
+        <v>530</v>
       </c>
     </row>
     <row r="9">
@@ -1000,16 +996,16 @@
         <v>32</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>16</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="10">
@@ -1025,16 +1021,16 @@
         <v>26</v>
       </c>
       <c r="D10" s="4" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E10" s="4" t="n">
         <v>13</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
     </row>
     <row r="11">
@@ -1050,16 +1046,16 @@
         <v>26</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E11" s="4" t="n">
         <v>13</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
     </row>
     <row r="12">
@@ -1075,16 +1071,16 @@
         <v>84</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>66</v>
+        <v>76</v>
       </c>
       <c r="E12" s="5" t="n">
         <v>42</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>16</v>
+        <v>30</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>284</v>
+        <v>308</v>
       </c>
     </row>
     <row r="13">
@@ -1100,16 +1096,16 @@
         <v>236</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>188</v>
+        <v>198</v>
       </c>
       <c r="E13" s="9" t="n">
         <v>120</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>42</v>
+        <v>70</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>800</v>
+        <v>838</v>
       </c>
     </row>
   </sheetData>
@@ -1199,13 +1195,13 @@
         <v>28</v>
       </c>
       <c r="E3" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F3" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G3" s="4" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
     </row>
     <row r="4">
@@ -1227,10 +1223,10 @@
         <v>11</v>
       </c>
       <c r="F4" s="4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G4" s="4" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="5">
@@ -1252,10 +1248,10 @@
         <v>16</v>
       </c>
       <c r="F5" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6">
@@ -1277,10 +1273,10 @@
         <v>12</v>
       </c>
       <c r="F6" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G6" s="4" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="7">
@@ -1299,13 +1295,13 @@
         <v>116</v>
       </c>
       <c r="E7" s="5" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="F7" s="5" t="n">
-        <v>20</v>
+        <v>36</v>
       </c>
       <c r="G7" s="5" t="n">
-        <v>404</v>
+        <v>422</v>
       </c>
     </row>
     <row r="9">
@@ -1315,22 +1311,22 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C9" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D9" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C9" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="D9" s="4" t="n">
-        <v>25</v>
-      </c>
       <c r="E9" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
     </row>
     <row r="10">
@@ -1340,22 +1336,22 @@
         </is>
       </c>
       <c r="B10" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C10" s="4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D10" s="4" t="n">
         <v>19</v>
       </c>
       <c r="E10" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="11">
@@ -1368,19 +1364,19 @@
         <v>18</v>
       </c>
       <c r="C11" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D11" s="4" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E11" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F11" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G11" s="4" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
     </row>
     <row r="12">
@@ -1390,22 +1386,22 @@
         </is>
       </c>
       <c r="B12" s="5" t="n">
-        <v>59</v>
+        <v>62</v>
       </c>
       <c r="C12" s="5" t="n">
-        <v>59</v>
+        <v>64</v>
       </c>
       <c r="D12" s="5" t="n">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E12" s="5" t="n">
-        <v>29</v>
+        <v>36</v>
       </c>
       <c r="F12" s="5" t="n">
-        <v>10</v>
+        <v>24</v>
       </c>
       <c r="G12" s="5" t="n">
-        <v>220</v>
+        <v>250</v>
       </c>
     </row>
     <row r="13">
@@ -1415,22 +1411,22 @@
         </is>
       </c>
       <c r="B13" s="9" t="n">
-        <v>167</v>
+        <v>170</v>
       </c>
       <c r="C13" s="9" t="n">
-        <v>168</v>
+        <v>173</v>
       </c>
       <c r="D13" s="9" t="n">
-        <v>179</v>
+        <v>180</v>
       </c>
       <c r="E13" s="9" t="n">
-        <v>80</v>
+        <v>89</v>
       </c>
       <c r="F13" s="9" t="n">
-        <v>30</v>
+        <v>60</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>624</v>
+        <v>672</v>
       </c>
     </row>
   </sheetData>
@@ -1468,7 +1464,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Caracas · 4 tiendas CCS (2 alto peso · 1 media · 1 bajo) · MC · Blanco + Azul Marino al 70%</t>
+          <t>Caracas · 4 tiendas CCS · MC · Blanco 283 + Azul Marino 209 · total 492</t>
         </is>
       </c>
     </row>
@@ -1536,16 +1532,16 @@
         <v>32</v>
       </c>
       <c r="D8" s="4" t="n">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="E8" s="4" t="n">
         <v>16</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>110</v>
+        <v>116</v>
       </c>
     </row>
     <row r="9">
@@ -1567,10 +1563,10 @@
         <v>23</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>156</v>
+        <v>158</v>
       </c>
     </row>
     <row r="10">
@@ -1586,16 +1582,16 @@
         <v>78</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>39</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>14</v>
+        <v>20</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>266</v>
+        <v>274</v>
       </c>
     </row>
     <row r="12">
@@ -1656,22 +1652,22 @@
         </is>
       </c>
       <c r="B15" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="C15" s="4" t="n">
+        <v>25</v>
+      </c>
+      <c r="D15" s="4" t="n">
         <v>23</v>
       </c>
-      <c r="C15" s="4" t="n">
-        <v>23</v>
-      </c>
-      <c r="D15" s="4" t="n">
-        <v>25</v>
-      </c>
       <c r="E15" s="4" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>4</v>
+        <v>8</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>86</v>
+        <v>93</v>
       </c>
     </row>
     <row r="16">
@@ -1693,10 +1689,10 @@
         <v>16</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="17">
@@ -1706,22 +1702,22 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="D17" s="5" t="n">
-        <v>60</v>
+        <v>58</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>209</v>
+        <v>218</v>
       </c>
     </row>
     <row r="19">
@@ -1731,7 +1727,7 @@
         </is>
       </c>
       <c r="B19" s="11" t="n">
-        <v>475</v>
+        <v>492</v>
       </c>
     </row>
   </sheetData>
@@ -1769,7 +1765,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Valencia · 2 tiendas · MC · Blanco + Vinotinto al 70%</t>
+          <t>Valencia · 2 tiendas · MC · Blanco 228 + Vinotinto 174 · total 402</t>
         </is>
       </c>
     </row>
@@ -1843,10 +1839,10 @@
         <v>19</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>124</v>
+        <v>128</v>
       </c>
     </row>
     <row r="9">
@@ -1862,16 +1858,16 @@
         <v>26</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>13</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10">
@@ -1887,16 +1883,16 @@
         <v>63</v>
       </c>
       <c r="D10" s="5" t="n">
-        <v>49</v>
+        <v>53</v>
       </c>
       <c r="E10" s="5" t="n">
         <v>32</v>
       </c>
       <c r="F10" s="5" t="n">
-        <v>11</v>
+        <v>20</v>
       </c>
       <c r="G10" s="5" t="n">
-        <v>211</v>
+        <v>224</v>
       </c>
     </row>
     <row r="12">
@@ -1969,10 +1965,10 @@
         <v>12</v>
       </c>
       <c r="F15" s="4" t="n">
-        <v>5</v>
+        <v>8</v>
       </c>
       <c r="G15" s="4" t="n">
-        <v>97</v>
+        <v>100</v>
       </c>
     </row>
     <row r="16">
@@ -1982,22 +1978,22 @@
         </is>
       </c>
       <c r="B16" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="C16" s="4" t="n">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="D16" s="4" t="n">
         <v>19</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>67</v>
+        <v>78</v>
       </c>
     </row>
     <row r="17">
@@ -2007,22 +2003,22 @@
         </is>
       </c>
       <c r="B17" s="5" t="n">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="C17" s="5" t="n">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="D17" s="5" t="n">
         <v>47</v>
       </c>
       <c r="E17" s="5" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F17" s="5" t="n">
-        <v>8</v>
+        <v>16</v>
       </c>
       <c r="G17" s="5" t="n">
-        <v>164</v>
+        <v>178</v>
       </c>
     </row>
     <row r="19">
@@ -2032,7 +2028,7 @@
         </is>
       </c>
       <c r="B19" s="11" t="n">
-        <v>375</v>
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -2070,7 +2066,7 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Barquisimeto · 1 tienda · MC · Ciudad 220 + Virgen 200 + Verde 154 (70% Ciudad) · total 574</t>
+          <t>Barquisimeto · 1 tienda · MC · Ciudad 231 + Virgen 210 + Verde 175 · total 616</t>
         </is>
       </c>
     </row>
@@ -2144,10 +2140,10 @@
         <v>19</v>
       </c>
       <c r="F8" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G8" s="4" t="n">
-        <v>123</v>
+        <v>127</v>
       </c>
     </row>
     <row r="9">
@@ -2163,16 +2159,16 @@
         <v>26</v>
       </c>
       <c r="D9" s="4" t="n">
-        <v>20</v>
+        <v>24</v>
       </c>
       <c r="E9" s="4" t="n">
         <v>13</v>
       </c>
       <c r="F9" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G9" s="4" t="n">
-        <v>87</v>
+        <v>96</v>
       </c>
     </row>
     <row r="10">
@@ -2194,10 +2190,10 @@
         <v>17</v>
       </c>
       <c r="F10" s="4" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="G10" s="4" t="n">
-        <v>113</v>
+        <v>117</v>
       </c>
     </row>
     <row r="11">
@@ -2213,16 +2209,16 @@
         <v>95</v>
       </c>
       <c r="D11" s="5" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="E11" s="5" t="n">
         <v>49</v>
       </c>
       <c r="F11" s="5" t="n">
-        <v>17</v>
+        <v>30</v>
       </c>
       <c r="G11" s="5" t="n">
-        <v>323</v>
+        <v>340</v>
       </c>
     </row>
     <row r="13">
@@ -2292,13 +2288,13 @@
         <v>28</v>
       </c>
       <c r="E16" s="4" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F16" s="4" t="n">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="G16" s="4" t="n">
-        <v>97</v>
+        <v>104</v>
       </c>
     </row>
     <row r="17">
@@ -2311,19 +2307,19 @@
         <v>18</v>
       </c>
       <c r="C17" s="4" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="D17" s="4" t="n">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E17" s="4" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F17" s="4" t="n">
-        <v>3</v>
+        <v>8</v>
       </c>
       <c r="G17" s="4" t="n">
-        <v>67</v>
+        <v>79</v>
       </c>
     </row>
     <row r="18">
@@ -2345,10 +2341,10 @@
         <v>11</v>
       </c>
       <c r="F18" s="4" t="n">
-        <v>4</v>
+        <v>10</v>
       </c>
       <c r="G18" s="4" t="n">
-        <v>87</v>
+        <v>93</v>
       </c>
     </row>
     <row r="19">
@@ -2361,19 +2357,19 @@
         <v>67</v>
       </c>
       <c r="C19" s="5" t="n">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="D19" s="5" t="n">
-        <v>72</v>
+        <v>75</v>
       </c>
       <c r="E19" s="5" t="n">
-        <v>32</v>
+        <v>37</v>
       </c>
       <c r="F19" s="5" t="n">
-        <v>12</v>
+        <v>28</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>251</v>
+        <v>276</v>
       </c>
     </row>
     <row r="21">
@@ -2383,7 +2379,7 @@
         </is>
       </c>
       <c r="B21" s="11" t="n">
-        <v>574</v>
+        <v>616</v>
       </c>
     </row>
   </sheetData>
@@ -2459,7 +2455,7 @@
         </is>
       </c>
       <c r="C4" s="4" t="n">
-        <v>920</v>
+        <v>952</v>
       </c>
       <c r="D4" s="4" t="inlineStr">
         <is>
@@ -2472,7 +2468,7 @@
         </is>
       </c>
       <c r="F4" s="4" t="n">
-        <v>497</v>
+        <v>514</v>
       </c>
     </row>
     <row r="5">
@@ -2487,7 +2483,7 @@
         </is>
       </c>
       <c r="C5" s="4" t="n">
-        <v>220</v>
+        <v>231</v>
       </c>
       <c r="D5" s="4" t="inlineStr">
         <is>
@@ -2500,7 +2496,7 @@
         </is>
       </c>
       <c r="F5" s="4" t="n">
-        <v>119</v>
+        <v>125</v>
       </c>
     </row>
     <row r="6">
@@ -2515,7 +2511,7 @@
         </is>
       </c>
       <c r="C6" s="4" t="n">
-        <v>200</v>
+        <v>210</v>
       </c>
       <c r="D6" s="4" t="inlineStr">
         <is>
@@ -2528,7 +2524,7 @@
         </is>
       </c>
       <c r="F6" s="4" t="n">
-        <v>108</v>
+        <v>113</v>
       </c>
     </row>
     <row r="7">
@@ -2543,7 +2539,7 @@
         </is>
       </c>
       <c r="C7" s="4" t="n">
-        <v>196</v>
+        <v>209</v>
       </c>
       <c r="D7" s="4" t="inlineStr">
         <is>
@@ -2556,7 +2552,7 @@
         </is>
       </c>
       <c r="F7" s="4" t="n">
-        <v>106</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8">
@@ -2571,7 +2567,7 @@
         </is>
       </c>
       <c r="C8" s="4" t="n">
-        <v>154</v>
+        <v>174</v>
       </c>
       <c r="D8" s="4" t="inlineStr">
         <is>
@@ -2584,7 +2580,7 @@
         </is>
       </c>
       <c r="F8" s="4" t="n">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="9">
@@ -2599,7 +2595,7 @@
         </is>
       </c>
       <c r="C9" s="4" t="n">
-        <v>154</v>
+        <v>175</v>
       </c>
       <c r="D9" s="4" t="inlineStr">
         <is>
@@ -2612,7 +2608,7 @@
         </is>
       </c>
       <c r="F9" s="4" t="n">
-        <v>83</v>
+        <v>94</v>
       </c>
     </row>
     <row r="10">
@@ -2627,7 +2623,7 @@
         </is>
       </c>
       <c r="C10" s="5" t="n">
-        <v>1424</v>
+        <v>1510</v>
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
@@ -2640,7 +2636,7 @@
         </is>
       </c>
       <c r="F10" s="5" t="n">
-        <v>769</v>
+        <v>815</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Sync SPOTS dashboard with manual production Excel (1,510 und / 815 kg)
- Add spots_produccion_manual.py to load CAB/DAMA from SPOTS_PRODUCCION_EXPANSION.xlsx
- Prefer manual expansion in rebuild_data when xlsx is present
- Regenerate dashboard with manual_xlsx source and adjusted zone totals
- Update CORREO draft totals to match synced production matrix

Co-authored-by: scm-svg <scm-svg@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/SPOTS_PRODUCCION_EXPANSION.xlsx
+++ b/SPOTS_PRODUCCION_EXPANSION.xlsx
@@ -532,7 +532,11 @@
           <t>Base rotación</t>
         </is>
       </c>
-      <c r="B4" t="inlineStr"/>
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Jun 26 · Jul 26 · Ago 26</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="2" t="inlineStr">
@@ -684,7 +688,7 @@
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>Cantidades ajustadas manualmente · horizonte 3 meses · colores: Caracas Azul Marino · Valencia Vinotinto · Barquisimeto Verde.</t>
+          <t>Cantidades ajustadas manualmente (SPOTS_PRODUCCION_EXPANSION.xlsx) · horizonte 3 meses · colores: Caracas Azul Marino · Valencia Vinotinto · Barquisimeto Verde. Total 1510 und. Base rotación VELA: Jun 26, Jul 26, Ago 26.</t>
         </is>
       </c>
     </row>

</xml_diff>